<commit_message>
Atualiza arquivos de métricas e gráficos de evolução do erro no Adaline
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -485,37 +485,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04289848953589559</v>
+        <v>0.2626014057250683</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1384538233415276</v>
+        <v>0.2871871684006001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5971753034935263</v>
+        <v>0.3338575251049209</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2997400420060883</v>
+        <v>0.5882550552644531</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9051355529908324</v>
+        <v>0.8308272863547894</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.811403147204154</v>
+        <v>-3.347172104590511</v>
       </c>
       <c r="H2" t="n">
-        <v>1.312533327780612</v>
+        <v>1.412348215366406</v>
       </c>
       <c r="I2" t="n">
-        <v>1.641370969343198</v>
+        <v>2.436285666939883</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.4266049181231152</v>
+        <v>-1.386788725558269</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.177123572857835</v>
+        <v>-1.538646608579109</v>
       </c>
       <c r="L2" t="n">
-        <v>874</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -525,37 +525,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3173566539875597</v>
+        <v>0.9567201037485323</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2868545494040374</v>
+        <v>0.509962280103854</v>
       </c>
       <c r="D3" t="n">
-        <v>0.787731605552535</v>
+        <v>0.143120648974568</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2280676519740199</v>
+        <v>0.9789099430268807</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9628657425999365</v>
+        <v>0.8147997191544624</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.81125162409968</v>
+        <v>-3.347172635044204</v>
       </c>
       <c r="H3" t="n">
-        <v>1.312527866998524</v>
+        <v>1.412348277457956</v>
       </c>
       <c r="I3" t="n">
-        <v>1.641318757223016</v>
+        <v>2.436285972620521</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.4264585693889776</v>
+        <v>-1.386789058649159</v>
       </c>
       <c r="K3" t="n">
-        <v>-1.177082957283175</v>
+        <v>-1.538646710447636</v>
       </c>
       <c r="L3" t="n">
-        <v>880</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -565,37 +565,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3978402639193718</v>
+        <v>0.3058556733530837</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5620282189080513</v>
+        <v>0.05970368903326551</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8070161698698157</v>
+        <v>0.6598244734142776</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01899217805759756</v>
+        <v>0.7068653136094304</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9853537168065982</v>
+        <v>0.3696872557621946</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.811267786774996</v>
+        <v>-3.347172771867048</v>
       </c>
       <c r="H4" t="n">
-        <v>1.312515061780266</v>
+        <v>1.412348463969301</v>
       </c>
       <c r="I4" t="n">
-        <v>1.641307488173511</v>
+        <v>2.436286096488377</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.4265008269318374</v>
+        <v>-1.38678927305905</v>
       </c>
       <c r="K4" t="n">
-        <v>-1.177077554027331</v>
+        <v>-1.538646728088736</v>
       </c>
       <c r="L4" t="n">
-        <v>874</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -605,37 +605,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1059012921808319</v>
+        <v>0.05130862864292351</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6590455163622504</v>
+        <v>0.9590187826489549</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7297376894335139</v>
+        <v>0.9034036494465233</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6908461407020068</v>
+        <v>0.1968832590027512</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3366958750227624</v>
+        <v>0.5139696484540538</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.81136516003324</v>
+        <v>-3.347172068455988</v>
       </c>
       <c r="H5" t="n">
-        <v>1.31263028301746</v>
+        <v>1.412347860277762</v>
       </c>
       <c r="I5" t="n">
-        <v>1.64148134186789</v>
+        <v>2.436285553423481</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.4263730102491579</v>
+        <v>-1.386788439144374</v>
       </c>
       <c r="K5" t="n">
-        <v>-1.177184778043431</v>
+        <v>-1.538646619264556</v>
       </c>
       <c r="L5" t="n">
-        <v>873</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -645,37 +645,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06357839535486198</v>
+        <v>0.2877417447815279</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6691488352469595</v>
+        <v>0.2894603032682652</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5468422114225763</v>
+        <v>0.1516425884942287</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8338838961013613</v>
+        <v>0.8022285208646371</v>
       </c>
       <c r="F6" t="n">
-        <v>0.716638132807061</v>
+        <v>0.6525621556607418</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.811269448376543</v>
+        <v>-3.347172110297067</v>
       </c>
       <c r="H6" t="n">
-        <v>1.312611516551508</v>
+        <v>1.412348285038999</v>
       </c>
       <c r="I6" t="n">
-        <v>1.641429136801486</v>
+        <v>2.436285688511409</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.4263109581264952</v>
+        <v>-1.386788780166252</v>
       </c>
       <c r="K6" t="n">
-        <v>-1.177148006568979</v>
+        <v>-1.538646606381641</v>
       </c>
       <c r="L6" t="n">
-        <v>888</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove previsão de classificação e atualiza arquivos de métricas e gráficos de evolução do erro no Adaline
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -485,37 +485,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2626014057250683</v>
+        <v>0.6216104340573222</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2871871684006001</v>
+        <v>0.1956662598928921</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3338575251049209</v>
+        <v>0.9031481827152088</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5882550552644531</v>
+        <v>0.9030638288601074</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8308272863547894</v>
+        <v>0.6634211027356375</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.347172104590511</v>
+        <v>-1.811323177047153</v>
       </c>
       <c r="H2" t="n">
-        <v>1.412348215366406</v>
+        <v>1.312639112838401</v>
       </c>
       <c r="I2" t="n">
-        <v>2.436285666939883</v>
+        <v>1.641479873439822</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.386788725558269</v>
+        <v>-0.4263118996767787</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.538646608579109</v>
+        <v>-1.177181040047292</v>
       </c>
       <c r="L2" t="n">
-        <v>51</v>
+        <v>912</v>
       </c>
     </row>
     <row r="3">
@@ -525,37 +525,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9567201037485323</v>
+        <v>0.6742232805293642</v>
       </c>
       <c r="C3" t="n">
-        <v>0.509962280103854</v>
+        <v>0.9977857066231026</v>
       </c>
       <c r="D3" t="n">
-        <v>0.143120648974568</v>
+        <v>0.7266045947383825</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9789099430268807</v>
+        <v>0.7238617934030919</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8147997191544624</v>
+        <v>0.2109037028366538</v>
       </c>
       <c r="G3" t="n">
-        <v>-3.347172635044204</v>
+        <v>-1.811344331411226</v>
       </c>
       <c r="H3" t="n">
-        <v>1.412348277457956</v>
+        <v>1.312660424605471</v>
       </c>
       <c r="I3" t="n">
-        <v>2.436285972620521</v>
+        <v>1.641512935695812</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.386789058649159</v>
+        <v>-0.4262916035224095</v>
       </c>
       <c r="K3" t="n">
-        <v>-1.538646710447636</v>
+        <v>-1.177201613286922</v>
       </c>
       <c r="L3" t="n">
-        <v>51</v>
+        <v>899</v>
       </c>
     </row>
     <row r="4">
@@ -565,37 +565,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3058556733530837</v>
+        <v>0.1825021321588147</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05970368903326551</v>
+        <v>0.9337294802802709</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6598244734142776</v>
+        <v>0.359072414351768</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7068653136094304</v>
+        <v>0.5473705463354778</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3696872557621946</v>
+        <v>0.9700603040589423</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.347172771867048</v>
+        <v>-1.811227255927235</v>
       </c>
       <c r="H4" t="n">
-        <v>1.412348463969301</v>
+        <v>1.312571253006767</v>
       </c>
       <c r="I4" t="n">
-        <v>2.436286096488377</v>
+        <v>1.641365926753693</v>
       </c>
       <c r="J4" t="n">
-        <v>-1.38678927305905</v>
+        <v>-0.4263471835616351</v>
       </c>
       <c r="K4" t="n">
-        <v>-1.538646728088736</v>
+        <v>-1.177108554978941</v>
       </c>
       <c r="L4" t="n">
-        <v>50</v>
+        <v>891</v>
       </c>
     </row>
     <row r="5">
@@ -605,37 +605,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05130862864292351</v>
+        <v>0.8630679339249526</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9590187826489549</v>
+        <v>0.8976087838291736</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9034036494465233</v>
+        <v>0.4186440750961156</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1968832590027512</v>
+        <v>0.2790369943143295</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5139696484540538</v>
+        <v>0.3940650821071694</v>
       </c>
       <c r="G5" t="n">
-        <v>-3.347172068455988</v>
+        <v>-1.811262940716975</v>
       </c>
       <c r="H5" t="n">
-        <v>1.412347860277762</v>
+        <v>1.31258405514835</v>
       </c>
       <c r="I5" t="n">
-        <v>2.436285553423481</v>
+        <v>1.64139267079435</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.386788439144374</v>
+        <v>-0.4263588150226914</v>
       </c>
       <c r="K5" t="n">
-        <v>-1.538646619264556</v>
+        <v>-1.177126474367147</v>
       </c>
       <c r="L5" t="n">
-        <v>51</v>
+        <v>904</v>
       </c>
     </row>
     <row r="6">
@@ -645,37 +645,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2877417447815279</v>
+        <v>0.1501348270879282</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2894603032682652</v>
+        <v>0.8819779953287229</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1516425884942287</v>
+        <v>0.4917366930618841</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8022285208646371</v>
+        <v>0.1365992570711146</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6525621556607418</v>
+        <v>0.5298157349227886</v>
       </c>
       <c r="G6" t="n">
-        <v>-3.347172110297067</v>
+        <v>-1.811363175812918</v>
       </c>
       <c r="H6" t="n">
-        <v>1.412348285038999</v>
+        <v>1.312541813822989</v>
       </c>
       <c r="I6" t="n">
-        <v>2.436285688511409</v>
+        <v>1.641369608074715</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.386788780166252</v>
+        <v>-0.4265467267976883</v>
       </c>
       <c r="K6" t="n">
-        <v>-1.538646606381641</v>
+        <v>-1.177120036522683</v>
       </c>
       <c r="L6" t="n">
-        <v>51</v>
+        <v>862</v>
       </c>
     </row>
   </sheetData>

</xml_diff>